<commit_message>
Mejoras en ETL Excel, UVS, etc.
Mejoras en como se extraen los datos de excel.
mejoras en el dashboard para visualizacion de UVs.
historial de solicitudes etc.
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_status_alumno.xlsx
+++ b/public/templates/plantilla_status_alumno.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Proyectos\Proyect-E\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7297C05C-DD42-4EC5-8648-2EC6C45EA4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C71F578-6E5D-4436-B3BC-19A3DAE7E9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="3075" windowWidth="16410" windowHeight="14145" xr2:uid="{9833ED06-4074-4667-99AE-6EF94282758F}"/>
+    <workbookView xWindow="30495" yWindow="-6900" windowWidth="12150" windowHeight="15585" xr2:uid="{9833ED06-4074-4667-99AE-6EF94282758F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$Y$45</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -28,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="137">
   <si>
     <t>cuenta</t>
   </si>
@@ -36,9 +40,6 @@
     <t>nombre</t>
   </si>
   <si>
-    <t>plan</t>
-  </si>
-  <si>
     <t>codigo_carrera</t>
   </si>
   <si>
@@ -100,13 +101,355 @@
   </si>
   <si>
     <t>orientacion</t>
+  </si>
+  <si>
+    <t>MAT101</t>
+  </si>
+  <si>
+    <t>INTRODUCCIÓN AL ÁLGEBRA</t>
+  </si>
+  <si>
+    <t>ADM102</t>
+  </si>
+  <si>
+    <t>ADMINISTRACIÓN I</t>
+  </si>
+  <si>
+    <t>APB</t>
+  </si>
+  <si>
+    <t>FIL101</t>
+  </si>
+  <si>
+    <t>FILOSOFÍA</t>
+  </si>
+  <si>
+    <t>BIO202</t>
+  </si>
+  <si>
+    <t>ECOLOGÍA</t>
+  </si>
+  <si>
+    <t>MAT102</t>
+  </si>
+  <si>
+    <t>ÁLGEBRA</t>
+  </si>
+  <si>
+    <t>REH302</t>
+  </si>
+  <si>
+    <t>GER.RECURSOS HUMANOS I</t>
+  </si>
+  <si>
+    <t>LCC104</t>
+  </si>
+  <si>
+    <t>OFIMÁTICA AVANZADA</t>
+  </si>
+  <si>
+    <t>ESP103</t>
+  </si>
+  <si>
+    <t>COMUNICACIÓN ORAL Y ESCRITA</t>
+  </si>
+  <si>
+    <t>REP</t>
+  </si>
+  <si>
+    <t>INF201</t>
+  </si>
+  <si>
+    <t>COMERCIO ELECTRÓNICO</t>
+  </si>
+  <si>
+    <t>EQV</t>
+  </si>
+  <si>
+    <t>CCC106</t>
+  </si>
+  <si>
+    <t>ART107</t>
+  </si>
+  <si>
+    <t>CCC104</t>
+  </si>
+  <si>
+    <t>DEP102</t>
+  </si>
+  <si>
+    <t>FIS201</t>
+  </si>
+  <si>
+    <t>FIS202</t>
+  </si>
+  <si>
+    <t>HIS101</t>
+  </si>
+  <si>
+    <t>MAT001</t>
+  </si>
+  <si>
+    <t>MAT103</t>
+  </si>
+  <si>
+    <t>MAT105</t>
+  </si>
+  <si>
+    <t>MAT109</t>
+  </si>
+  <si>
+    <t>MAT203</t>
+  </si>
+  <si>
+    <t>MAT210</t>
+  </si>
+  <si>
+    <t>MAT301</t>
+  </si>
+  <si>
+    <t>SOC101</t>
+  </si>
+  <si>
+    <t>CCC105</t>
+  </si>
+  <si>
+    <t>CCC208</t>
+  </si>
+  <si>
+    <t>CCC217</t>
+  </si>
+  <si>
+    <t>CCC218</t>
+  </si>
+  <si>
+    <t>ADM103</t>
+  </si>
+  <si>
+    <t>MAT303</t>
+  </si>
+  <si>
+    <t>CCC301</t>
+  </si>
+  <si>
+    <t>CCC401</t>
+  </si>
+  <si>
+    <t>INF308</t>
+  </si>
+  <si>
+    <t>TEL201</t>
+  </si>
+  <si>
+    <t>INF309</t>
+  </si>
+  <si>
+    <t>CCC310</t>
+  </si>
+  <si>
+    <t>CCC308</t>
+  </si>
+  <si>
+    <t>CON319</t>
+  </si>
+  <si>
+    <t>CCC109</t>
+  </si>
+  <si>
+    <t>CCC412</t>
+  </si>
+  <si>
+    <t>CCC311</t>
+  </si>
+  <si>
+    <t>INF501</t>
+  </si>
+  <si>
+    <t>CCC413</t>
+  </si>
+  <si>
+    <t>Ceutec Sap</t>
+  </si>
+  <si>
+    <t>88.00</t>
+  </si>
+  <si>
+    <t>93.00</t>
+  </si>
+  <si>
+    <t>INTRODUCCIÓN COMPUTACIÓN</t>
+  </si>
+  <si>
+    <t>100.00</t>
+  </si>
+  <si>
+    <t>APRECIACIÓN LITERARIA</t>
+  </si>
+  <si>
+    <t>- -</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN I</t>
+  </si>
+  <si>
+    <t>BALONCESTO</t>
+  </si>
+  <si>
+    <t>FÍSICA I</t>
+  </si>
+  <si>
+    <t>FISICA II</t>
+  </si>
+  <si>
+    <t>HISTORIA DE HONDURAS</t>
+  </si>
+  <si>
+    <t>MATEMÁTICA NIVELATORIA</t>
+  </si>
+  <si>
+    <t>GEOMETRÍA TRIGONOMETRÍA</t>
+  </si>
+  <si>
+    <t>ÁLGEBRA LINEAL</t>
+  </si>
+  <si>
+    <t>CÁLCULO I</t>
+  </si>
+  <si>
+    <t>ECUACIONES DIFERENC.</t>
+  </si>
+  <si>
+    <t>CÁLCULO II</t>
+  </si>
+  <si>
+    <t>ESTADÍST. MATEMÁTICA I</t>
+  </si>
+  <si>
+    <t>SOCIOLOGÍA</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN II</t>
+  </si>
+  <si>
+    <t>70.00</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN III</t>
+  </si>
+  <si>
+    <t>60.00</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN WEB</t>
+  </si>
+  <si>
+    <t>91.00</t>
+  </si>
+  <si>
+    <t>PROGRAMACIÓN MÓVIL</t>
+  </si>
+  <si>
+    <t>89.00</t>
+  </si>
+  <si>
+    <t>V5483</t>
+  </si>
+  <si>
+    <t>ADMINISTRACIÓN II</t>
+  </si>
+  <si>
+    <t>48.00</t>
+  </si>
+  <si>
+    <t>MATEMATICAS DISCRETAS</t>
+  </si>
+  <si>
+    <t>80.00</t>
+  </si>
+  <si>
+    <t>ESTRUCTURA DE DATOS</t>
+  </si>
+  <si>
+    <t>95.00</t>
+  </si>
+  <si>
+    <t>90.00</t>
+  </si>
+  <si>
+    <t>SISTEMAS OPERATIVOS I</t>
+  </si>
+  <si>
+    <t>92.00</t>
+  </si>
+  <si>
+    <t>ADMINISTRACIÓN BASE DE DATOS I</t>
+  </si>
+  <si>
+    <t>REDES</t>
+  </si>
+  <si>
+    <t>ADMINISTRACIÓN BASE DATOS II</t>
+  </si>
+  <si>
+    <t>72.00</t>
+  </si>
+  <si>
+    <t>CIENCIA DE DATOS I</t>
+  </si>
+  <si>
+    <t>83.00</t>
+  </si>
+  <si>
+    <t>INGENIERÍA DE SOFTWARE I</t>
+  </si>
+  <si>
+    <t>82.00</t>
+  </si>
+  <si>
+    <t>CONTABILIDAD GERENCIAL</t>
+  </si>
+  <si>
+    <t>74.00</t>
+  </si>
+  <si>
+    <t>ÉTICA INFORMÁTICA</t>
+  </si>
+  <si>
+    <t>INGENIERÍA DE SOFTWARE II</t>
+  </si>
+  <si>
+    <t>97.00</t>
+  </si>
+  <si>
+    <t>CIENCIA DE DATOS II</t>
+  </si>
+  <si>
+    <t>84.00</t>
+  </si>
+  <si>
+    <t>0.00</t>
+  </si>
+  <si>
+    <t>AUDITORÍA INFORMÁTICA</t>
+  </si>
+  <si>
+    <t>16.00</t>
+  </si>
+  <si>
+    <t>DESARROLLO APLICAC. VANGUARDIA</t>
+  </si>
+  <si>
+    <t>IdPlan</t>
+  </si>
+  <si>
+    <t>AnioPlan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,8 +465,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF212121"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -136,8 +485,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -145,15 +500,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFE0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="15" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -470,35 +854,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E9F1FC-91D5-42D4-B6F1-34D8E7CC5484}">
-  <dimension ref="A1:X45"/>
+  <dimension ref="A1:Y45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,73 +892,76 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -582,23 +971,24 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="J2" s="4"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+      <c r="L2" s="5"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
+      <c r="R2" s="7"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
+      <c r="V2" s="9"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y2" s="3"/>
+    </row>
+    <row r="3" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -608,23 +998,24 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="J3" s="4"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
+      <c r="L3" s="5"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="R3" s="7"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
+      <c r="V3" s="9"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y3" s="3"/>
+    </row>
+    <row r="4" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -634,23 +1025,24 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
+      <c r="L4" s="5"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+      <c r="R4" s="7"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
+      <c r="V4" s="9"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y4" s="3"/>
+    </row>
+    <row r="5" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -660,23 +1052,24 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="J5" s="4"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
+      <c r="L5" s="5"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
+      <c r="R5" s="7"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
+      <c r="V5" s="9"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y5" s="3"/>
+    </row>
+    <row r="6" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -686,23 +1079,24 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="J6" s="4"/>
       <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
+      <c r="L6" s="5"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
+      <c r="R6" s="7"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
+      <c r="V6" s="9"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y6" s="3"/>
+    </row>
+    <row r="7" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -712,23 +1106,24 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="J7" s="4"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
+      <c r="L7" s="5"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
+      <c r="R7" s="7"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
+      <c r="V7" s="9"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y7" s="3"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -738,23 +1133,24 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="J8" s="4"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
+      <c r="L8" s="5"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
+      <c r="R8" s="7"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
-      <c r="V8" s="3"/>
+      <c r="V8" s="9"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y8" s="3"/>
+    </row>
+    <row r="9" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -764,23 +1160,24 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="J9" s="4"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="L9" s="5"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
+      <c r="R9" s="7"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
+      <c r="V9" s="9"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y9" s="3"/>
+    </row>
+    <row r="10" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -790,23 +1187,24 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="J10" s="4"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+      <c r="L10" s="5"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
+      <c r="R10" s="7"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
+      <c r="V10" s="9"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y10" s="3"/>
+    </row>
+    <row r="11" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -816,23 +1214,24 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="J11" s="4"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
+      <c r="L11" s="5"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
+      <c r="R11" s="7"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
+      <c r="V11" s="9"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y11" s="3"/>
+    </row>
+    <row r="12" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -842,23 +1241,24 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="J12" s="4"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
+      <c r="L12" s="5"/>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
+      <c r="R12" s="7"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
+      <c r="V12" s="9"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y12" s="3"/>
+    </row>
+    <row r="13" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -868,23 +1268,24 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
+      <c r="J13" s="4"/>
       <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
+      <c r="L13" s="5"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
+      <c r="R13" s="7"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
+      <c r="V13" s="9"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y13" s="3"/>
+    </row>
+    <row r="14" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -894,23 +1295,24 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
+      <c r="J14" s="4"/>
       <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
+      <c r="L14" s="5"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
+      <c r="R14" s="7"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
+      <c r="V14" s="9"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y14" s="3"/>
+    </row>
+    <row r="15" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -920,23 +1322,24 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="J15" s="4"/>
       <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="L15" s="5"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
+      <c r="R15" s="7"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
+      <c r="V15" s="9"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y15" s="3"/>
+    </row>
+    <row r="16" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -946,23 +1349,24 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
+      <c r="J16" s="4"/>
       <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
+      <c r="L16" s="5"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
+      <c r="R16" s="7"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
-      <c r="V16" s="3"/>
+      <c r="V16" s="9"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y16" s="3"/>
+    </row>
+    <row r="17" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -972,23 +1376,24 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
+      <c r="J17" s="4"/>
       <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+      <c r="L17" s="5"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
       <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
+      <c r="R17" s="7"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
+      <c r="V17" s="9"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y17" s="3"/>
+    </row>
+    <row r="18" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -998,23 +1403,24 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
+      <c r="J18" s="4"/>
       <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+      <c r="L18" s="5"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
+      <c r="R18" s="7"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
+      <c r="V18" s="9"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y18" s="3"/>
+    </row>
+    <row r="19" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1024,23 +1430,24 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="J19" s="4"/>
       <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
+      <c r="L19" s="5"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
+      <c r="R19" s="7"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
+      <c r="V19" s="9"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y19" s="3"/>
+    </row>
+    <row r="20" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1050,23 +1457,24 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
+      <c r="J20" s="4"/>
       <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
+      <c r="L20" s="5"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
+      <c r="R20" s="7"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
-      <c r="V20" s="3"/>
+      <c r="V20" s="9"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y20" s="3"/>
+    </row>
+    <row r="21" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1076,23 +1484,24 @@
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+      <c r="J21" s="4"/>
       <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
+      <c r="L21" s="5"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
-      <c r="R21" s="3"/>
+      <c r="R21" s="7"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
-      <c r="V21" s="3"/>
+      <c r="V21" s="9"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y21" s="3"/>
+    </row>
+    <row r="22" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1102,23 +1511,24 @@
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
+      <c r="J22" s="4"/>
       <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
+      <c r="L22" s="5"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
-      <c r="R22" s="3"/>
+      <c r="R22" s="7"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
-      <c r="V22" s="3"/>
+      <c r="V22" s="9"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y22" s="3"/>
+    </row>
+    <row r="23" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1128,23 +1538,24 @@
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
+      <c r="J23" s="4"/>
       <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
+      <c r="L23" s="5"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
-      <c r="R23" s="3"/>
+      <c r="R23" s="7"/>
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
-      <c r="V23" s="3"/>
+      <c r="V23" s="9"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y23" s="3"/>
+    </row>
+    <row r="24" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1154,23 +1565,24 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
+      <c r="J24" s="4"/>
       <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
+      <c r="L24" s="5"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
-      <c r="R24" s="3"/>
+      <c r="R24" s="7"/>
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
-      <c r="V24" s="3"/>
+      <c r="V24" s="9"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y24" s="3"/>
+    </row>
+    <row r="25" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1180,23 +1592,24 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
+      <c r="J25" s="4"/>
       <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
+      <c r="L25" s="5"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
-      <c r="R25" s="3"/>
+      <c r="R25" s="7"/>
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
-      <c r="V25" s="3"/>
+      <c r="V25" s="9"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y25" s="3"/>
+    </row>
+    <row r="26" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1206,23 +1619,24 @@
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
+      <c r="J26" s="4"/>
       <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
+      <c r="L26" s="5"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
+      <c r="R26" s="7"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
-      <c r="V26" s="3"/>
+      <c r="V26" s="9"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y26" s="3"/>
+    </row>
+    <row r="27" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1232,23 +1646,24 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
+      <c r="J27" s="4"/>
       <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
+      <c r="L27" s="5"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
-      <c r="R27" s="3"/>
+      <c r="R27" s="7"/>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
-      <c r="V27" s="3"/>
+      <c r="V27" s="9"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y27" s="3"/>
+    </row>
+    <row r="28" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1258,23 +1673,24 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
+      <c r="J28" s="4"/>
       <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
+      <c r="L28" s="5"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
+      <c r="R28" s="7"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
-      <c r="V28" s="3"/>
+      <c r="V28" s="9"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y28" s="3"/>
+    </row>
+    <row r="29" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1284,23 +1700,24 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
+      <c r="J29" s="4"/>
       <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
+      <c r="L29" s="5"/>
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
-      <c r="R29" s="3"/>
+      <c r="R29" s="7"/>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
-      <c r="V29" s="3"/>
+      <c r="V29" s="9"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y29" s="3"/>
+    </row>
+    <row r="30" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1310,23 +1727,24 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
+      <c r="J30" s="4"/>
       <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
+      <c r="L30" s="5"/>
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
-      <c r="R30" s="3"/>
+      <c r="R30" s="7"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
-      <c r="V30" s="3"/>
+      <c r="V30" s="9"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y30" s="3"/>
+    </row>
+    <row r="31" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1336,23 +1754,24 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
+      <c r="J31" s="4"/>
       <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
+      <c r="L31" s="5"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
-      <c r="R31" s="3"/>
+      <c r="R31" s="7"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
-      <c r="V31" s="3"/>
+      <c r="V31" s="9"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y31" s="3"/>
+    </row>
+    <row r="32" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1362,23 +1781,24 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
+      <c r="J32" s="4"/>
       <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
+      <c r="L32" s="5"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
-      <c r="R32" s="3"/>
+      <c r="R32" s="7"/>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
-      <c r="V32" s="3"/>
+      <c r="V32" s="9"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y32" s="3"/>
+    </row>
+    <row r="33" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1388,23 +1808,24 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
+      <c r="J33" s="4"/>
       <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
+      <c r="L33" s="5"/>
       <c r="M33" s="3"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
-      <c r="R33" s="3"/>
+      <c r="R33" s="7"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
-      <c r="V33" s="3"/>
+      <c r="V33" s="9"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y33" s="3"/>
+    </row>
+    <row r="34" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1414,23 +1835,24 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
+      <c r="J34" s="4"/>
       <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
+      <c r="L34" s="5"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
-      <c r="R34" s="3"/>
+      <c r="R34" s="7"/>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
-      <c r="V34" s="3"/>
+      <c r="V34" s="9"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y34" s="3"/>
+    </row>
+    <row r="35" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1440,23 +1862,24 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
+      <c r="J35" s="4"/>
       <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
+      <c r="L35" s="5"/>
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
-      <c r="R35" s="3"/>
+      <c r="R35" s="7"/>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
-      <c r="V35" s="3"/>
+      <c r="V35" s="9"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y35" s="3"/>
+    </row>
+    <row r="36" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1466,23 +1889,24 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
+      <c r="J36" s="4"/>
       <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
+      <c r="L36" s="5"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
-      <c r="R36" s="3"/>
+      <c r="R36" s="7"/>
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
-      <c r="V36" s="3"/>
+      <c r="V36" s="9"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
-    </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y36" s="3"/>
+    </row>
+    <row r="37" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1492,23 +1916,24 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
+      <c r="J37" s="4"/>
       <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
+      <c r="L37" s="5"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
-      <c r="R37" s="3"/>
+      <c r="R37" s="7"/>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
-      <c r="V37" s="3"/>
+      <c r="V37" s="9"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
-    </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y37" s="3"/>
+    </row>
+    <row r="38" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1518,23 +1943,24 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
+      <c r="J38" s="4"/>
       <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
+      <c r="L38" s="5"/>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
       <c r="Q38" s="3"/>
-      <c r="R38" s="3"/>
+      <c r="R38" s="7"/>
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
-      <c r="V38" s="3"/>
+      <c r="V38" s="9"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y38" s="3"/>
+    </row>
+    <row r="39" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1544,23 +1970,24 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
+      <c r="J39" s="4"/>
       <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
+      <c r="L39" s="5"/>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
-      <c r="R39" s="3"/>
+      <c r="R39" s="7"/>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
-      <c r="V39" s="3"/>
+      <c r="V39" s="9"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y39" s="3"/>
+    </row>
+    <row r="40" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1570,23 +1997,24 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
+      <c r="J40" s="4"/>
       <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
+      <c r="L40" s="5"/>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
-      <c r="R40" s="3"/>
+      <c r="R40" s="7"/>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
-      <c r="V40" s="3"/>
+      <c r="V40" s="9"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y40" s="3"/>
+    </row>
+    <row r="41" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1596,23 +2024,24 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
+      <c r="J41" s="4"/>
       <c r="K41" s="3"/>
-      <c r="L41" s="3"/>
+      <c r="L41" s="5"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
-      <c r="R41" s="3"/>
+      <c r="R41" s="7"/>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
-      <c r="V41" s="3"/>
+      <c r="V41" s="9"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
-    </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y41" s="3"/>
+    </row>
+    <row r="42" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1622,23 +2051,24 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
+      <c r="J42" s="4"/>
       <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
+      <c r="L42" s="5"/>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
-      <c r="R42" s="3"/>
+      <c r="R42" s="7"/>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
-      <c r="V42" s="3"/>
+      <c r="V42" s="9"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
-    </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y42" s="3"/>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1648,9 +2078,9 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
+      <c r="J43" s="4"/>
       <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
+      <c r="L43" s="5"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
       <c r="O43" s="3"/>
@@ -1660,11 +2090,12 @@
       <c r="S43" s="3"/>
       <c r="T43" s="3"/>
       <c r="U43" s="3"/>
-      <c r="V43" s="3"/>
+      <c r="V43" s="9"/>
       <c r="W43" s="3"/>
       <c r="X43" s="3"/>
-    </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y43" s="3"/>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1674,9 +2105,9 @@
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
+      <c r="J44" s="4"/>
       <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
+      <c r="L44" s="5"/>
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
       <c r="O44" s="3"/>
@@ -1686,11 +2117,12 @@
       <c r="S44" s="3"/>
       <c r="T44" s="3"/>
       <c r="U44" s="3"/>
-      <c r="V44" s="3"/>
+      <c r="V44" s="9"/>
       <c r="W44" s="3"/>
       <c r="X44" s="3"/>
-    </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y44" s="3"/>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1700,9 +2132,9 @@
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
+      <c r="J45" s="4"/>
       <c r="K45" s="3"/>
-      <c r="L45" s="3"/>
+      <c r="L45" s="6"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
       <c r="O45" s="3"/>
@@ -1712,9 +2144,1434 @@
       <c r="S45" s="3"/>
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
-      <c r="V45" s="3"/>
+      <c r="V45" s="9"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
+      <c r="Y45" s="3"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y45" xr:uid="{20E9F1FC-91D5-42D4-B6F1-34D8E7CC5484}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106C6B0F-3F25-4780-A949-6F38D9871DF8}">
+  <dimension ref="A1:J44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C1" s="7">
+        <v>1</v>
+      </c>
+      <c r="D1" s="7">
+        <v>2</v>
+      </c>
+      <c r="E1" s="7">
+        <v>1339</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C2" s="7">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7">
+        <v>2</v>
+      </c>
+      <c r="E2" s="7">
+        <v>796</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C3" s="7">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7">
+        <v>4</v>
+      </c>
+      <c r="E3" s="7">
+        <v>154</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C4" s="7">
+        <v>2</v>
+      </c>
+      <c r="D4" s="7">
+        <v>4</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C5" s="7">
+        <v>2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C6" s="7">
+        <v>2</v>
+      </c>
+      <c r="D6" s="7">
+        <v>4</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="7">
+        <v>4</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2</v>
+      </c>
+      <c r="D8" s="7">
+        <v>4</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C9" s="7">
+        <v>2</v>
+      </c>
+      <c r="D9" s="7">
+        <v>4</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C10" s="7">
+        <v>2</v>
+      </c>
+      <c r="D10" s="7">
+        <v>4</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C11" s="7">
+        <v>2</v>
+      </c>
+      <c r="D11" s="7">
+        <v>4</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C12" s="7">
+        <v>2</v>
+      </c>
+      <c r="D12" s="7">
+        <v>4</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C13" s="7">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7">
+        <v>4</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C14" s="7">
+        <v>2</v>
+      </c>
+      <c r="D14" s="7">
+        <v>4</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J14" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C15" s="7">
+        <v>2</v>
+      </c>
+      <c r="D15" s="7">
+        <v>4</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J15" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C16" s="7">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7">
+        <v>4</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J16" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C17" s="7">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7">
+        <v>4</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C18" s="7">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7">
+        <v>4</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J18" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C19" s="7">
+        <v>2</v>
+      </c>
+      <c r="D19" s="7">
+        <v>4</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J19" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C20" s="7">
+        <v>2</v>
+      </c>
+      <c r="D20" s="7">
+        <v>4</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J20" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2</v>
+      </c>
+      <c r="D21" s="7">
+        <v>4</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J21" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C22" s="7">
+        <v>2</v>
+      </c>
+      <c r="D22" s="7">
+        <v>4</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J22" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C23" s="7">
+        <v>2</v>
+      </c>
+      <c r="D23" s="7">
+        <v>5</v>
+      </c>
+      <c r="E23" s="7">
+        <v>1011</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C24" s="7">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7">
+        <v>1</v>
+      </c>
+      <c r="E24" s="7">
+        <v>153</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B25" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C25" s="7">
+        <v>1</v>
+      </c>
+      <c r="D25" s="7">
+        <v>2</v>
+      </c>
+      <c r="E25" s="7">
+        <v>899</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C26" s="7">
+        <v>2</v>
+      </c>
+      <c r="D26" s="7">
+        <v>4</v>
+      </c>
+      <c r="E26" s="7">
+        <v>5</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C27" s="7">
+        <v>2</v>
+      </c>
+      <c r="D27" s="7">
+        <v>4</v>
+      </c>
+      <c r="E27" s="7">
+        <v>65</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C28" s="7">
+        <v>2</v>
+      </c>
+      <c r="D28" s="7">
+        <v>4</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J28" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C29" s="7">
+        <v>2</v>
+      </c>
+      <c r="D29" s="7">
+        <v>5</v>
+      </c>
+      <c r="E29" s="7">
+        <v>1286</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="7">
+        <v>2024</v>
+      </c>
+      <c r="C30" s="7">
+        <v>2</v>
+      </c>
+      <c r="D30" s="7">
+        <v>5</v>
+      </c>
+      <c r="E30" s="7">
+        <v>782</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J30" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C31" s="7">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7">
+        <v>1</v>
+      </c>
+      <c r="E31" s="7">
+        <v>177</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C32" s="7">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7">
+        <v>1</v>
+      </c>
+      <c r="E32" s="7">
+        <v>69</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C33" s="7">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7">
+        <v>1</v>
+      </c>
+      <c r="E33" s="7">
+        <v>71</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C34" s="7">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7">
+        <v>2</v>
+      </c>
+      <c r="E34" s="7">
+        <v>1285</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C35" s="7">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7">
+        <v>2</v>
+      </c>
+      <c r="E35" s="7">
+        <v>690</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C36" s="7">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7">
+        <v>4</v>
+      </c>
+      <c r="E36" s="7">
+        <v>1352</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J36" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C37" s="7">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7">
+        <v>4</v>
+      </c>
+      <c r="E37" s="7">
+        <v>1370</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J37" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C38" s="7">
+        <v>2</v>
+      </c>
+      <c r="D38" s="7">
+        <v>4</v>
+      </c>
+      <c r="E38" s="7">
+        <v>1693</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J38" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C39" s="7">
+        <v>2</v>
+      </c>
+      <c r="D39" s="7">
+        <v>5</v>
+      </c>
+      <c r="E39" s="7">
+        <v>166</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J39" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C40" s="7">
+        <v>2</v>
+      </c>
+      <c r="D40" s="7">
+        <v>5</v>
+      </c>
+      <c r="E40" s="7">
+        <v>233</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C41" s="7">
+        <v>2</v>
+      </c>
+      <c r="D41" s="7">
+        <v>5</v>
+      </c>
+      <c r="E41" s="7">
+        <v>234</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J41" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C42" s="7">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7">
+        <v>1</v>
+      </c>
+      <c r="E42" s="7">
+        <v>473</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="I42" s="7"/>
+      <c r="J42" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C43" s="7">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7">
+        <v>1</v>
+      </c>
+      <c r="E43" s="7">
+        <v>87</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C44" s="8">
+        <v>1</v>
+      </c>
+      <c r="D44" s="8">
+        <v>1</v>
+      </c>
+      <c r="E44" s="8">
+        <v>91</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="I44" s="8"/>
+      <c r="J44" s="8">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>